<commit_message>
frontend converted to react-router-dom v6.4.3, added a new component for the registration page, and added a new component for the ticket table. Also added a new component for the shell and page header. Added a new component for the icon. Added a new component for the logo. Added a new component for the field icon. Added a new component for the ticket table. Added a new component for the shell and page header. Added a new component for the icon. Added a new component for the logo. Added a new component for the field icon.
</commit_message>
<xml_diff>
--- a/docs/SmartDesk_UserStories_TaskPlan.xlsx
+++ b/docs/SmartDesk_UserStories_TaskPlan.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jh1\Desktop\smartdesk\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_A1FD566DF9301CD55D1EBD06489E0136361617B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="User Stories" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Task Plan &amp; Timeline" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="User Stories" sheetId="1" r:id="rId1"/>
+    <sheet name="Task Plan &amp; Timeline" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -23,542 +28,539 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="176">
   <si>
-    <t xml:space="preserve">Story ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use Case</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Actor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User Story</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acceptance Criteria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Story Points</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-01 Register Account</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employee/User</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a new user, I want to register with my name, email, and password so that I can access SmartDesk.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duplicate emails rejected; password securely hashed; success confirmation returned.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-02 Login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employee/Agent/Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a registered user, I want to log in so that I receive an authenticated session and land on my role's dashboard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valid credentials return a token; invalid credentials return a controlled error; role determines redirect.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authorization (FR 5.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As the system, I want to enforce role-based authorization so that users only access permitted actions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Protected endpoints reject unauthenticated/unauthorized requests; roles checked server-side.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-03 Create Ticket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an employee, I want to create a ticket with a title and description so IT can help me.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ticket saved with status OPEN; validation errors block bad input; AI analysis triggered when enabled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-04 View Own Tickets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an employee, I want to view my own tickets so I can track their progress.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">List shows only the employee's tickets with status/priority/category/dates; empty state when none exist.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-05 View Ticket Details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an authorized user, I want to view full ticket details so I understand its current state.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shows metadata, comments, assignment, status, and AI info where available; unauthorized users get an error.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-07 Assign Ticket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT Agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an IT agent, I want to assign a ticket to myself or another agent so ownership is clear.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only authorized assignees accepted; ticket appears in assignee's workload.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-08 Update Ticket Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an IT agent, I want to update ticket status and priority so the ticket reflects its real progress.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status limited to OPEN/IN_PROGRESS/RESOLVED; invalid transitions rejected; update timestamp recorded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-09 Add Ticket Comment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employee/IT Agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a ticket participant, I want to add comments so I can communicate updates.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comments store author/timestamp/content; shown chronologically; empty comments rejected.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-10 Resolve Ticket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an IT agent, I want to resolve a ticket so the employee knows their issue is fixed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status set to RESOLVED; resolution timestamp recorded; employee can see resolved state.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-06 Analyze Ticket with AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System/IT Agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As the system, I want to send a new ticket's description to the AI service so it gets classified automatically.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI returns category, priority, summary, suggested actions; malformed/failed AI responses don't block ticket creation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-06 Analyze Ticket with AI (review)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an IT agent, I want to review AI suggestions on a ticket before acting on them.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI analysis displayed on ticket details; agent can proceed with or override the suggestion.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Should</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-11 View Dashboard Statistics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT Agent/Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an IT agent or admin, I want to see ticket statistics so I can monitor service-desk activity.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard shows counts by status, category, and priority; empty/zero states handled gracefully.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-11 View Dashboard Statistics (workload)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an admin, I want to see agent workload so I can balance ticket assignment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard lists agents with open/assigned ticket counts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-12 Manage Users</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an admin, I want to view and manage user accounts so I can maintain the system.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin-only access; permitted attributes/role changes validated and saved.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC-13 Manage Categories</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an admin, I want to create and edit ticket categories so tickets stay well organized.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duplicate/invalid categories rejected; new category becomes available for tickets.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API Documentation (NFR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Developer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want Swagger/OpenAPI docs so the frontend can integrate against a clear contract.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swagger UI lists all endpoints with request/response schemas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testability (NFR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want automated backend tests so core logic is protected against regressions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUnit/Mockito cover auth, ticket, and AI services; Postman collection covers main endpoints.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deployability - Docker (NFR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the app containerized so it runs consistently across environments.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dockerfiles for frontend/backend; docker-compose runs frontend+backend+MySQL locally.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deployability - Azure (Section 11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the MVP deployed to Azure so it's accessible outside my machine.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend and backend reachable over HTTPS on Azure; backend connects to managed DB; secrets via Azure config.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finalization (Section 12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want polished documentation and a demo-ready build so I can present SmartDesk confidently.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">README, architecture/ER diagrams, and a working demo script are complete; deployment verified end-to-end.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint Focus (per SRS Sec. 12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daily Tasks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deliverable / Exit Criteria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Related Stories</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wednesday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project setup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Init Git repo; scaffold Spring Boot project; scaffold React project; create MySQL schema; set up initial architecture and environment configuration.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repos created; base backend/frontend run locally; DB reachable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thursday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authentication (part 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User entity + repository; registration endpoint; password hashing (BCrypt); Spring Security base config.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User can register via API with hashed password stored.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authentication (part 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login endpoint; JWT issuing/validation; role field on User; protected route middleware.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User can log in and receive a JWT; protected endpoint rejects missing/invalid token.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-02, US-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core ticket system (part 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ticket + Category entities and relationships; create-ticket endpoint; list-tickets endpoint scoped by role.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employee can create and list tickets via API.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tuesday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core ticket system (part 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ticket details endpoint; assign-ticket endpoint; update status/priority endpoint; resolve-ticket logic with resolved_at timestamp.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agent can view, assign, update status/priority, and resolve a ticket via API.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-06, US-07, US-08, US-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend MVP (part 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login page; Register page; Auth context + protected routes; Employee Dashboard shell; Agent Dashboard shell.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User can log in through the UI and land on the correct dashboard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-02, US-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend MVP (part 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ticket list page; Create Ticket page; Ticket Details page (status/assignment/AI panel placeholders).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employee can create/view tickets end-to-end in the UI.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-04, US-05, US-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comments + validation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comment entity + endpoints; comment UI on ticket details; Jakarta Validation on key DTOs; global exception handler; ticket filtering (status/category/priority).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comments work end-to-end; invalid input returns consistent error responses; ticket list is filterable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI integration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spring AI + OpenAI setup; ticket analysis service (category, priority, summary, suggested actions); graceful fallback if AI fails.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New tickets get AI-suggested category/priority/summary; agent can view and override it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-11, US-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard + API documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard statistics endpoint (by status/category/priority, agent workload); React dashboard UI; Swagger/OpenAPI setup; minor UI refinement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard shows live stats; all endpoints visible and testable in Swagger UI.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-13, US-14, US-15, US-16, US-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUnit/Mockito tests for auth, ticket, and AI services; Postman collection; basic security/integration checks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core services covered by automated tests; Postman collection runs cleanly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docker + Azure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dockerfiles for backend/frontend; docker-compose for local dev; Azure hosting setup for frontend/backend; managed DB; env/secrets via Azure config; enable HTTPS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docker-compose up runs the stack locally; app is reachable and functional on Azure over HTTPS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-19, US-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finalization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bug fixes; README; architecture and ER diagrams; demo script and screenshots; final deployment verification (frontend↔backend↔DB on Azure).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repo and live demo are presentation-ready.</t>
+    <t>Story ID</t>
+  </si>
+  <si>
+    <t>Use Case</t>
+  </si>
+  <si>
+    <t>Actor</t>
+  </si>
+  <si>
+    <t>User Story</t>
+  </si>
+  <si>
+    <t>Acceptance Criteria</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Story Points</t>
+  </si>
+  <si>
+    <t>Target Date</t>
+  </si>
+  <si>
+    <t>US-01</t>
+  </si>
+  <si>
+    <t>UC-01 Register Account</t>
+  </si>
+  <si>
+    <t>Employee/User</t>
+  </si>
+  <si>
+    <t>As a new user, I want to register with my name, email, and password so that I can access SmartDesk.</t>
+  </si>
+  <si>
+    <t>Duplicate emails rejected; password securely hashed; success confirmation returned.</t>
+  </si>
+  <si>
+    <t>Must</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>2026-09-03</t>
+  </si>
+  <si>
+    <t>US-02</t>
+  </si>
+  <si>
+    <t>UC-02 Login</t>
+  </si>
+  <si>
+    <t>Employee/Agent/Admin</t>
+  </si>
+  <si>
+    <t>As a registered user, I want to log in so that I receive an authenticated session and land on my role's dashboard.</t>
+  </si>
+  <si>
+    <t>Valid credentials return a token; invalid credentials return a controlled error; role determines redirect.</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>US-03</t>
+  </si>
+  <si>
+    <t>Authorization (FR 5.1)</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>As the system, I want to enforce role-based authorization so that users only access permitted actions.</t>
+  </si>
+  <si>
+    <t>Protected endpoints reject unauthenticated/unauthorized requests; roles checked server-side.</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>US-04</t>
+  </si>
+  <si>
+    <t>UC-03 Create Ticket</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>As an employee, I want to create a ticket with a title and description so IT can help me.</t>
+  </si>
+  <si>
+    <t>Ticket saved with status OPEN; validation errors block bad input; AI analysis triggered when enabled.</t>
+  </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
+    <t>US-05</t>
+  </si>
+  <si>
+    <t>UC-04 View Own Tickets</t>
+  </si>
+  <si>
+    <t>As an employee, I want to view my own tickets so I can track their progress.</t>
+  </si>
+  <si>
+    <t>List shows only the employee's tickets with status/priority/category/dates; empty state when none exist.</t>
+  </si>
+  <si>
+    <t>2026-09-09</t>
+  </si>
+  <si>
+    <t>US-06</t>
+  </si>
+  <si>
+    <t>UC-05 View Ticket Details</t>
+  </si>
+  <si>
+    <t>As an authorized user, I want to view full ticket details so I understand its current state.</t>
+  </si>
+  <si>
+    <t>Shows metadata, comments, assignment, status, and AI info where available; unauthorized users get an error.</t>
+  </si>
+  <si>
+    <t>2026-09-08</t>
+  </si>
+  <si>
+    <t>US-07</t>
+  </si>
+  <si>
+    <t>UC-07 Assign Ticket</t>
+  </si>
+  <si>
+    <t>IT Agent</t>
+  </si>
+  <si>
+    <t>As an IT agent, I want to assign a ticket to myself or another agent so ownership is clear.</t>
+  </si>
+  <si>
+    <t>Only authorized assignees accepted; ticket appears in assignee's workload.</t>
+  </si>
+  <si>
+    <t>US-08</t>
+  </si>
+  <si>
+    <t>UC-08 Update Ticket Status</t>
+  </si>
+  <si>
+    <t>As an IT agent, I want to update ticket status and priority so the ticket reflects its real progress.</t>
+  </si>
+  <si>
+    <t>Status limited to OPEN/IN_PROGRESS/RESOLVED; invalid transitions rejected; update timestamp recorded.</t>
+  </si>
+  <si>
+    <t>US-09</t>
+  </si>
+  <si>
+    <t>UC-09 Add Ticket Comment</t>
+  </si>
+  <si>
+    <t>Employee/IT Agent</t>
+  </si>
+  <si>
+    <t>As a ticket participant, I want to add comments so I can communicate updates.</t>
+  </si>
+  <si>
+    <t>Comments store author/timestamp/content; shown chronologically; empty comments rejected.</t>
+  </si>
+  <si>
+    <t>2026-09-11</t>
+  </si>
+  <si>
+    <t>US-10</t>
+  </si>
+  <si>
+    <t>UC-10 Resolve Ticket</t>
+  </si>
+  <si>
+    <t>As an IT agent, I want to resolve a ticket so the employee knows their issue is fixed.</t>
+  </si>
+  <si>
+    <t>Status set to RESOLVED; resolution timestamp recorded; employee can see resolved state.</t>
+  </si>
+  <si>
+    <t>US-11</t>
+  </si>
+  <si>
+    <t>UC-06 Analyze Ticket with AI</t>
+  </si>
+  <si>
+    <t>System/IT Agent</t>
+  </si>
+  <si>
+    <t>As the system, I want to send a new ticket's description to the AI service so it gets classified automatically.</t>
+  </si>
+  <si>
+    <t>AI returns category, priority, summary, suggested actions; malformed/failed AI responses don't block ticket creation.</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>US-12</t>
+  </si>
+  <si>
+    <t>UC-06 Analyze Ticket with AI (review)</t>
+  </si>
+  <si>
+    <t>As an IT agent, I want to review AI suggestions on a ticket before acting on them.</t>
+  </si>
+  <si>
+    <t>AI analysis displayed on ticket details; agent can proceed with or override the suggestion.</t>
+  </si>
+  <si>
+    <t>Should</t>
+  </si>
+  <si>
+    <t>US-13</t>
+  </si>
+  <si>
+    <t>UC-11 View Dashboard Statistics</t>
+  </si>
+  <si>
+    <t>IT Agent/Admin</t>
+  </si>
+  <si>
+    <t>As an IT agent or admin, I want to see ticket statistics so I can monitor service-desk activity.</t>
+  </si>
+  <si>
+    <t>Dashboard shows counts by status, category, and priority; empty/zero states handled gracefully.</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
+  </si>
+  <si>
+    <t>US-14</t>
+  </si>
+  <si>
+    <t>UC-11 View Dashboard Statistics (workload)</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>As an admin, I want to see agent workload so I can balance ticket assignment.</t>
+  </si>
+  <si>
+    <t>Dashboard lists agents with open/assigned ticket counts.</t>
+  </si>
+  <si>
+    <t>US-15</t>
+  </si>
+  <si>
+    <t>UC-12 Manage Users</t>
+  </si>
+  <si>
+    <t>As an admin, I want to view and manage user accounts so I can maintain the system.</t>
+  </si>
+  <si>
+    <t>Admin-only access; permitted attributes/role changes validated and saved.</t>
+  </si>
+  <si>
+    <t>US-16</t>
+  </si>
+  <si>
+    <t>UC-13 Manage Categories</t>
+  </si>
+  <si>
+    <t>As an admin, I want to create and edit ticket categories so tickets stay well organized.</t>
+  </si>
+  <si>
+    <t>Duplicate/invalid categories rejected; new category becomes available for tickets.</t>
+  </si>
+  <si>
+    <t>US-17</t>
+  </si>
+  <si>
+    <t>API Documentation (NFR)</t>
+  </si>
+  <si>
+    <t>Developer</t>
+  </si>
+  <si>
+    <t>As a developer, I want Swagger/OpenAPI docs so the frontend can integrate against a clear contract.</t>
+  </si>
+  <si>
+    <t>Swagger UI lists all endpoints with request/response schemas.</t>
+  </si>
+  <si>
+    <t>US-18</t>
+  </si>
+  <si>
+    <t>Testability (NFR)</t>
+  </si>
+  <si>
+    <t>As a developer, I want automated backend tests so core logic is protected against regressions.</t>
+  </si>
+  <si>
+    <t>JUnit/Mockito cover auth, ticket, and AI services; Postman collection covers main endpoints.</t>
+  </si>
+  <si>
+    <t>2026-09-16</t>
+  </si>
+  <si>
+    <t>US-19</t>
+  </si>
+  <si>
+    <t>Deployability - Docker (NFR)</t>
+  </si>
+  <si>
+    <t>As a developer, I want the app containerized so it runs consistently across environments.</t>
+  </si>
+  <si>
+    <t>Dockerfiles for frontend/backend; docker-compose runs frontend+backend+MySQL locally.</t>
+  </si>
+  <si>
+    <t>2026-09-17</t>
+  </si>
+  <si>
+    <t>US-20</t>
+  </si>
+  <si>
+    <t>Deployability - Azure (Section 11)</t>
+  </si>
+  <si>
+    <t>As a developer, I want the MVP deployed to Azure so it's accessible outside my machine.</t>
+  </si>
+  <si>
+    <t>Frontend and backend reachable over HTTPS on Azure; backend connects to managed DB; secrets via Azure config.</t>
+  </si>
+  <si>
+    <t>US-21</t>
+  </si>
+  <si>
+    <t>Finalization (Section 12)</t>
+  </si>
+  <si>
+    <t>As a developer, I want polished documentation and a demo-ready build so I can present SmartDesk confidently.</t>
+  </si>
+  <si>
+    <t>README, architecture/ER diagrams, and a working demo script are complete; deployment verified end-to-end.</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Weekday</t>
+  </si>
+  <si>
+    <t>Sprint Focus (per SRS Sec. 12)</t>
+  </si>
+  <si>
+    <t>Daily Tasks</t>
+  </si>
+  <si>
+    <t>Deliverable / Exit Criteria</t>
+  </si>
+  <si>
+    <t>Related Stories</t>
+  </si>
+  <si>
+    <t>2026-09-02</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>Project setup</t>
+  </si>
+  <si>
+    <t>Init Git repo; scaffold Spring Boot project; scaffold React project; create MySQL schema; set up initial architecture and environment configuration.</t>
+  </si>
+  <si>
+    <t>Repos created; base backend/frontend run locally; DB reachable.</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>Authentication (part 1)</t>
+  </si>
+  <si>
+    <t>User entity + repository; registration endpoint; password hashing (BCrypt); Spring Security base config.</t>
+  </si>
+  <si>
+    <t>User can register via API with hashed password stored.</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Authentication (part 2)</t>
+  </si>
+  <si>
+    <t>Login endpoint; JWT issuing/validation; role field on User; protected route middleware.</t>
+  </si>
+  <si>
+    <t>User can log in and receive a JWT; protected endpoint rejects missing/invalid token.</t>
+  </si>
+  <si>
+    <t>US-02, US-03</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>Core ticket system (part 1)</t>
+  </si>
+  <si>
+    <t>Ticket + Category entities and relationships; create-ticket endpoint; list-tickets endpoint scoped by role.</t>
+  </si>
+  <si>
+    <t>Employee can create and list tickets via API.</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>Core ticket system (part 2)</t>
+  </si>
+  <si>
+    <t>Ticket details endpoint; assign-ticket endpoint; update status/priority endpoint; resolve-ticket logic with resolved_at timestamp.</t>
+  </si>
+  <si>
+    <t>Agent can view, assign, update status/priority, and resolve a ticket via API.</t>
+  </si>
+  <si>
+    <t>US-06, US-07, US-08, US-10</t>
+  </si>
+  <si>
+    <t>Frontend MVP (part 1)</t>
+  </si>
+  <si>
+    <t>Login page; Register page; Auth context + protected routes; Employee Dashboard shell; Agent Dashboard shell.</t>
+  </si>
+  <si>
+    <t>User can log in through the UI and land on the correct dashboard.</t>
+  </si>
+  <si>
+    <t>US-02, US-05</t>
+  </si>
+  <si>
+    <t>2026-09-10</t>
+  </si>
+  <si>
+    <t>Frontend MVP (part 2)</t>
+  </si>
+  <si>
+    <t>Ticket list page; Create Ticket page; Ticket Details page (status/assignment/AI panel placeholders).</t>
+  </si>
+  <si>
+    <t>Employee can create/view tickets end-to-end in the UI.</t>
+  </si>
+  <si>
+    <t>US-04, US-05, US-06</t>
+  </si>
+  <si>
+    <t>Comments + validation</t>
+  </si>
+  <si>
+    <t>Comment entity + endpoints; comment UI on ticket details; Jakarta Validation on key DTOs; global exception handler; ticket filtering (status/category/priority).</t>
+  </si>
+  <si>
+    <t>Comments work end-to-end; invalid input returns consistent error responses; ticket list is filterable.</t>
+  </si>
+  <si>
+    <t>AI integration</t>
+  </si>
+  <si>
+    <t>Spring AI + OpenAI setup; ticket analysis service (category, priority, summary, suggested actions); graceful fallback if AI fails.</t>
+  </si>
+  <si>
+    <t>New tickets get AI-suggested category/priority/summary; agent can view and override it.</t>
+  </si>
+  <si>
+    <t>US-11, US-12</t>
+  </si>
+  <si>
+    <t>Dashboard + API documentation</t>
+  </si>
+  <si>
+    <t>Dashboard statistics endpoint (by status/category/priority, agent workload); React dashboard UI; Swagger/OpenAPI setup; minor UI refinement.</t>
+  </si>
+  <si>
+    <t>Dashboard shows live stats; all endpoints visible and testable in Swagger UI.</t>
+  </si>
+  <si>
+    <t>US-13, US-14, US-15, US-16, US-17</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>JUnit/Mockito tests for auth, ticket, and AI services; Postman collection; basic security/integration checks.</t>
+  </si>
+  <si>
+    <t>Core services covered by automated tests; Postman collection runs cleanly.</t>
+  </si>
+  <si>
+    <t>Docker + Azure</t>
+  </si>
+  <si>
+    <t>Dockerfiles for backend/frontend; docker-compose for local dev; Azure hosting setup for frontend/backend; managed DB; env/secrets via Azure config; enable HTTPS.</t>
+  </si>
+  <si>
+    <t>docker-compose up runs the stack locally; app is reachable and functional on Azure over HTTPS.</t>
+  </si>
+  <si>
+    <t>US-19, US-20</t>
+  </si>
+  <si>
+    <t>Finalization</t>
+  </si>
+  <si>
+    <t>Bug fixes; README; architecture and ER diagrams; demo script and screenshots; final deployment verification (frontend↔backend↔DB on Azure).</t>
+  </si>
+  <si>
+    <t>Repo and live demo are presentation-ready.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -567,32 +569,15 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -617,14 +602,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFBFBFBF"/>
       </left>
@@ -640,57 +625,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -749,47 +703,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -797,12 +767,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -831,7 +801,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -852,7 +822,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -903,7 +873,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -921,33 +891,32 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="6" max="6" width="9" customWidth="1"/>
+    <col min="7" max="7" width="8" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -973,7 +942,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -999,7 +968,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>16</v>
       </c>
@@ -1025,7 +994,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -1051,7 +1020,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>28</v>
       </c>
@@ -1077,7 +1046,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
@@ -1103,7 +1072,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>39</v>
       </c>
@@ -1129,7 +1098,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>44</v>
       </c>
@@ -1155,7 +1124,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>49</v>
       </c>
@@ -1181,7 +1150,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>53</v>
       </c>
@@ -1207,7 +1176,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>59</v>
       </c>
@@ -1233,7 +1202,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>63</v>
       </c>
@@ -1259,7 +1228,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>69</v>
       </c>
@@ -1285,7 +1254,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>74</v>
       </c>
@@ -1311,7 +1280,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>80</v>
       </c>
@@ -1337,7 +1306,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>85</v>
       </c>
@@ -1363,7 +1332,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
@@ -1389,7 +1358,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>93</v>
       </c>
@@ -1415,7 +1384,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>98</v>
       </c>
@@ -1441,7 +1410,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>103</v>
       </c>
@@ -1467,7 +1436,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>108</v>
       </c>
@@ -1493,7 +1462,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>112</v>
       </c>
@@ -1520,33 +1489,25 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:6" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>117</v>
       </c>
@@ -1566,7 +1527,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>123</v>
       </c>
@@ -1584,7 +1545,7 @@
       </c>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -1604,7 +1565,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -1624,7 +1585,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>33</v>
       </c>
@@ -1644,7 +1605,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>43</v>
       </c>
@@ -1664,7 +1625,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>38</v>
       </c>
@@ -1684,7 +1645,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>150</v>
       </c>
@@ -1704,7 +1665,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>58</v>
       </c>
@@ -1724,7 +1685,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>68</v>
       </c>
@@ -1744,7 +1705,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>79</v>
       </c>
@@ -1764,7 +1725,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>102</v>
       </c>
@@ -1784,7 +1745,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>107</v>
       </c>
@@ -1804,7 +1765,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:6" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>116</v>
       </c>
@@ -1825,12 +1786,7 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added role based notification and fixed the avatar intials on the comments it was showing only intilas of the ticket creator.
</commit_message>
<xml_diff>
--- a/docs/SmartDesk_UserStories_TaskPlan.xlsx
+++ b/docs/SmartDesk_UserStories_TaskPlan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jh1\Desktop\smartdesk\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_A1FD566DF9301CD55D1EBD06489E0136361617B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44CDC01-5E2D-4B38-9A0C-E20D2A2DA04E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -581,7 +581,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -598,6 +598,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -628,7 +640,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -637,6 +649,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -943,262 +961,262 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="4" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="5" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1255,106 +1273,106 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="4" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="4" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="H17" s="5" t="s">
         <v>79</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed reset password functionality used form password
</commit_message>
<xml_diff>
--- a/docs/SmartDesk_UserStories_TaskPlan.xlsx
+++ b/docs/SmartDesk_UserStories_TaskPlan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jh1\Desktop\smartdesk\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44CDC01-5E2D-4B38-9A0C-E20D2A2DA04E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{916E21C0-B38C-4E30-8AC8-3B46AF35B3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Stories" sheetId="1" r:id="rId1"/>
@@ -1221,54 +1221,54 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="5" t="s">
         <v>68</v>
       </c>
     </row>

</xml_diff>